<commit_message>
docs: plan.js 입력·출력의 빈칸 확정, 명세 v17 (N19·N20)
</commit_message>
<xml_diff>
--- a/docs/spec.xlsx
+++ b/docs/spec.xlsx
@@ -53,7 +53,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2026-10-29 · v16 (v2: </t>
+      <t xml:space="preserve">2026-11-02 · v17 (v2: </t>
     </r>
     <r>
       <rPr>
@@ -1141,7 +1141,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(N24, F10-07) / v15: hasFavicon의 출력을 true·false에서 쓸 파비콘 주소 또는 null로 바꿈. 첫 페이지 주소에서 찾았을 때 appIcon이 그 주소로 그리게 함(N07, N44) / v16: N14 setPending 입력 필드 이름을 { id, toParentId }로 확정)</t>
+      <t xml:space="preserve">(N24, F10-07) / v15: hasFavicon의 출력을 true·false에서 쓸 파비콘 주소 또는 null로 바꿈. 첫 페이지 주소에서 찾았을 때 appIcon이 그 주소로 그리게 함(N07, N44) / v16: N14 setPending 입력 필드 이름을 { id, toParentId }로 확정 / v17: N19·N20 입력·출력의 빈칸 확정. N19 options의 키 이름과 기본값, 제외 조건(javascript:·chrome:// 주소, manualMoves의 키) / N20 reasons는 폴더 안, rest는 개수, pin의 reason은 "tooFew"·"noGroup", 폴더 순서(이슈 #11))</t>
     </r>
   </si>
   <si>
@@ -17259,13 +17259,13 @@
     <t xml:space="preserve">getTargets(tree, stored, options, now)</t>
   </si>
   <si>
-    <t xml:space="preserve">북마크 목록, 저장 항목, {북마크바 제외, 포함할 사용자 폴더}, 현재 시각</t>
-  </si>
-  <si>
-    <t xml:space="preserve">정리 대상 북마크 배열</t>
-  </si>
-  <si>
-    <t xml:space="preserve">북마크바·기타·모바일과 크롬 가져오기 폴더의 바로 아래에 흩어진 북마크를 고르고 제외 대상(사용자 폴더, 최근 30일 안에 북마크바에서 연 북마크, 직접 옮긴 북마크 등)을 뺌</t>
+    <t xml:space="preserve">북마크 목록, 저장 항목, { excludeBar, includeFolderIds }(북마크바 제외, 포함할 사용자 폴더 ID 배열. 기본값 { excludeBar: false, includeFolderIds: [] }), 현재 시각</t>
+  </si>
+  <si>
+    <t xml:space="preserve">정리 대상 북마크 배열(loadTree의 북마크 객체, tree.bookmarks의 순서 그대로)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">북마크바·기타·모바일과 크롬 가져오기 폴더의 바로 아래에 흩어진 북마크를 고르고 제외 대상(사용자 폴더, 최근 30일 안에 북마크바에서 연 북마크, javascript:·chrome:// 주소, 직접 옮긴 북마크)을 뺌</t>
   </si>
   <si>
     <r>
@@ -17830,6 +17830,16 @@
       </rPr>
       <t xml:space="preserve">그런 폴더는 사용자 폴더로 취급되어 정리 대상에서 빠진다</t>
     </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+v17: 직접 옮긴 북마크는 stored.manualMoves의 키(북마크 ID)로 판단. 요즘 쓰는 북마크는 rootType이 "bar"이고 dateLastUsed가 있으며 now - dateLastUsed &lt; 30일인 것(잊고 있던 북마크의 30일 이상과 겹치지 않게 "미만"). options를 안 넘기거나 일부만 넘기면 기본값을 씀. excludeBar: true면 북마크바 바로 아래의 북마크만 빼고, 가져오기 폴더("가져온 북마크") 바로 아래의 북마크는 그대로 둠(HTML을 가져오면 대부분이 그 폴더에 들어가기 때문). includeFolderIds는 그 폴더의 바로 아래 북마크만 넣고(하위 폴더는 넣지 않음), 관리 폴더(managed)와 고르지 않은 루트(rootChosen: false)의 폴더는 무시함. options는 F06-04(P2)에서 씀</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">#11</t>
@@ -17851,72 +17861,22 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">{ type: "folders", folders: [{name, items, reasons}], rest } </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">또는 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">{ type: "pin", reason }</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">개수에 맞는 폴더 수를 정하고, 많은 카테고리부터 폴더로 계획</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개 미만이거나 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개 이상 모인 카테고리가 없으면 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">type: "pin"</t>
+      <t xml:space="preserve">{ type: "folders", folders: [{ name, items, reasons }], rest } 또는 { type: "pin", reason }. name: 카테고리 이름, items: 북마크 객체 배열(targets의 순서), reasons: [{ bookmarkId, step, rule, needsCheck }](items와 같은 순서·같은 길이), rest: 폴더에 들어가지 않은 정리 대상의 개수(숫자), reason: "tooFew" | "noGroup"</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">개수에 맞는 폴더 수를 정하고, 많은 카테고리부터 폴더로 계획. folders는 북마크가 많은 순, 개수가 같으면 categories.json에 적힌 순서</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">정리 대상이 10개 미만이면 { type: "pin", reason: "tooFew" }, 10개 이상이지만 3개 이상 모인 카테고리가 없으면 { type: "pin", reason: "noGroup" }. reason은 화면에 그대로 보여 주지 않고, 문구는 cards.js가 F09-01대로 씀
+v17: 폴더 수 상한은 F05-05(10~29개 3, 30~59개 4, 60~99개 5, 100개 이상 6), 3개 미만 카테고리 제외와 "기타" 폴더 없음은 F05-06, 분류 안 됨은 폴더에 넣지 않음(F05-08). rest는 분류 안 됨, 3개 미만 카테고리, 상한 밖의 카테고리를 모두 셈. reasons는 classify의 출력에서 category를 빼고 bookmarkId를 붙인 것(F06-03 분류 근거, F06-05 "확인 필요"는 needsCheck)</t>
     </r>
   </si>
   <si>

</xml_diff>